<commit_message>
feat: add linktree module and update WhatsApp links to api.whatsapp.com format
</commit_message>
<xml_diff>
--- a/linktree/template/planilha_naturalmente_pronta.xlsx
+++ b/linktree/template/planilha_naturalmente_pronta.xlsx
@@ -41,7 +41,7 @@
     <t>Agendar avaliação gratuita</t>
   </si>
   <si>
-    <t>https://wa.me/5516992133717?text=Ol%C3%A1%2C%20Dra.%20Carolina%21%20Vim%20pelo%20link%20e%20gostaria%20de%20agendar%20minha%20avalia%C3%A7%C3%A3o%20%E2%9C%A8</t>
+    <t>https://api.whatsapp.com/send?phone=5516992133717&amp;text=Ol%C3%A1%2C%20Dra.%20Carolina%21%20Vim%20pelo%20link%20e%20gostaria%20de%20agendar%20minha%20avalia%C3%A7%C3%A3o%20%E2%9C%A8</t>
   </si>
   <si>
     <t>Site oficial</t>
@@ -83,7 +83,7 @@
     <t>whatsapp</t>
   </si>
   <si>
-    <t>https://wa.me/5516992133717</t>
+    <t>https://api.whatsapp.com/send?phone=5516992133717</t>
   </si>
   <si>
     <t>subtitulo</t>

</xml_diff>